<commit_message>
update pentest token remediation evidence
</commit_message>
<xml_diff>
--- a/docs/security/2026-Cashsouk-Web-Application-Grey-Box-remediated.xlsx
+++ b/docs/security/2026-Cashsouk-Web-Application-Grey-Box-remediated.xlsx
@@ -680,7 +680,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11.5" customWidth="1" min="1" max="1"/>
     <col width="25.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -886,7 +886,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="6.33203125" customWidth="1" min="1" max="1"/>
     <col width="17.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="L3" s="29" t="inlineStr">
         <is>
-          <t>21 Sep 2026: Added a PostgreSQL-backed access-token jti denylist with expiry cleanup, enforced by requireAuth. Both logout routes revoke the current access token before local teardown and then perform Cognito global sign-out; revocation-store failures fail closed with HTTP 503. Tokens issued at or before password_changed_at are also rejected. Portal logout only clears the local session after backend revocation succeeds. Prisma migration 20260921140000_revoked_access_tokens must run before the new API task is deployed.</t>
+          <t>21 Sep 2026: Added a PostgreSQL-backed access-token jti denylist with expiry cleanup, enforced by requireAuth. Both logout routes persist access-token revocation before local teardown, perform Cognito global sign-out, explicitly revoke the current browser httpOnly refresh token through Cognito RevokeToken, and clear that refresh cookie only after successful/idempotent revocation. Denylist or Cognito revocation failures fail closed with HTTP 503 and preserve local auth for retry. Password changes compare Cognito auth_time (falling back to iat), so an old refresh token cannot restore API access by minting a JWT with a newer iat. Prisma migration 20260921140000_revoked_access_tokens must run before the new API task is deployed.</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="L5" s="29" t="inlineStr">
         <is>
-          <t>21 Sep 2026: Centralized a shared password policy for API and all portal change-password/admin-user forms: minimum 8 characters, upper/lower case, number, a Cognito-supported symbol, and a common-password denylist. Cognito already enforces length/complexity, so the user pool was not changed. Password changes invalidate access tokens using password_changed_at and Cognito global sign-out.</t>
+          <t>21 Sep 2026: Centralized a shared password policy for API and all portal change-password/admin-user forms: minimum 8 characters, upper/lower case, number, a Cognito-supported symbol, and a common-password denylist. Cognito already enforces length/complexity, so the user pool was not changed. Password changes invalidate tokens authenticated at or before password_changed_at using Cognito auth_time, while Cognito global sign-out and explicit refresh-token revocation prevent session renewal.</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="25.1640625" bestFit="1" customWidth="1" min="2" max="2"/>

</xml_diff>